<commit_message>
updated spani population figures to include 2026 data
</commit_message>
<xml_diff>
--- a/data_demography/INE total and foreign population figures Spain.xlsx
+++ b/data_demography/INE total and foreign population figures Spain.xlsx
@@ -8,9 +8,9 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="INE_Foreign_population" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="INE_Total_population" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="INE_Total_foreign_population" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="INE_Foreign_population" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="INE_Total_population" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="INE_Total_foreign_population" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="253">
   <si>
     <t xml:space="preserve">Total Nacional. Extranjera. Todas las edades. Total. Población. Número. </t>
   </si>
@@ -769,6 +769,9 @@
   </si>
   <si>
     <t xml:space="preserve">Foreign Total YoY)(%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 de enero de 2026</t>
   </si>
   <si>
     <t xml:space="preserve">1 de enero de 2025</t>
@@ -1163,6 +1166,112 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -1674,8 +1783,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Página &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -3906,7 +4015,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.27"/>
@@ -3968,14 +4077,14 @@
         <v>249</v>
       </c>
       <c r="B4" s="20" t="n">
-        <v>49077984</v>
+        <v>49596376</v>
       </c>
       <c r="C4" s="20" t="n">
-        <v>6852348</v>
+        <v>7256796</v>
       </c>
       <c r="D4" s="24" t="n">
         <f aca="false">(C4/B4)</f>
-        <v>0.139621627489833</v>
+        <v>0.146317061553046</v>
       </c>
       <c r="E4" s="23"/>
       <c r="F4" s="23"/>
@@ -3984,693 +4093,724 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>25</v>
+        <v>250</v>
       </c>
       <c r="B5" s="20" t="n">
-        <v>48619695</v>
+        <v>49128297</v>
       </c>
       <c r="C5" s="20" t="n">
-        <v>6502282</v>
+        <v>6911971</v>
       </c>
       <c r="D5" s="24" t="n">
         <f aca="false">(C5/B5)</f>
-        <v>0.133737613944308</v>
+        <v>0.140692257254511</v>
       </c>
       <c r="E5" s="23" t="n">
         <f aca="false">B4-B5</f>
-        <v>458289</v>
+        <v>468079</v>
       </c>
       <c r="F5" s="25" t="n">
         <f aca="false">(B4-B5)/B5</f>
-        <v>0.00942599495945008</v>
+        <v>0.0095276862538101</v>
       </c>
       <c r="G5" s="23" t="n">
         <f aca="false">C4-C5</f>
-        <v>350066</v>
+        <v>344825</v>
       </c>
       <c r="H5" s="25" t="n">
         <f aca="false">(C4-C5)/C5</f>
-        <v>0.0538374066212447</v>
+        <v>0.0498880854679512</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B6" s="20" t="n">
-        <v>48085361</v>
+        <v>48619695</v>
       </c>
       <c r="C6" s="20" t="n">
-        <v>6089620</v>
+        <v>6502282</v>
       </c>
       <c r="D6" s="24" t="n">
         <f aca="false">(C6/B6)</f>
-        <v>0.1266418692375</v>
+        <v>0.133737613944308</v>
       </c>
       <c r="E6" s="23" t="n">
         <f aca="false">B5-B6</f>
-        <v>534334</v>
+        <v>508602</v>
       </c>
       <c r="F6" s="25" t="n">
         <f aca="false">(B5-B6)/B6</f>
-        <v>0.0111121969116547</v>
+        <v>0.0104608225123584</v>
       </c>
       <c r="G6" s="23" t="n">
         <f aca="false">C5-C6</f>
-        <v>412662</v>
+        <v>409689</v>
       </c>
       <c r="H6" s="25" t="n">
         <f aca="false">(C5-C6)/C6</f>
-        <v>0.0677648194797048</v>
+        <v>0.0630069566346092</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B7" s="20" t="n">
-        <v>47486727</v>
+        <v>48085361</v>
       </c>
       <c r="C7" s="20" t="n">
-        <v>5509046</v>
+        <v>6089620</v>
       </c>
       <c r="D7" s="24" t="n">
         <f aca="false">(C7/B7)</f>
-        <v>0.116012333298945</v>
+        <v>0.1266418692375</v>
       </c>
       <c r="E7" s="23" t="n">
         <f aca="false">B6-B7</f>
-        <v>598634</v>
+        <v>534334</v>
       </c>
       <c r="F7" s="25" t="n">
         <f aca="false">(B6-B7)/B7</f>
-        <v>0.0126063436631461</v>
+        <v>0.0111121969116547</v>
       </c>
       <c r="G7" s="23" t="n">
         <f aca="false">C6-C7</f>
-        <v>580574</v>
+        <v>412662</v>
       </c>
       <c r="H7" s="25" t="n">
         <f aca="false">(C6-C7)/C7</f>
-        <v>0.105385578555706</v>
+        <v>0.0677648194797048</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B8" s="20" t="n">
-        <v>47400798</v>
+        <v>47486727</v>
       </c>
       <c r="C8" s="20" t="n">
-        <v>5402702</v>
+        <v>5509046</v>
       </c>
       <c r="D8" s="24" t="n">
         <f aca="false">(C8/B8)</f>
-        <v>0.11397913596307</v>
+        <v>0.116012333298945</v>
       </c>
       <c r="E8" s="23" t="n">
         <f aca="false">B7-B8</f>
-        <v>85929</v>
+        <v>598634</v>
       </c>
       <c r="F8" s="25" t="n">
         <f aca="false">(B7-B8)/B8</f>
-        <v>0.00181281758167869</v>
+        <v>0.0126063436631461</v>
       </c>
       <c r="G8" s="23" t="n">
         <f aca="false">C7-C8</f>
-        <v>106344</v>
+        <v>580574</v>
       </c>
       <c r="H8" s="25" t="n">
         <f aca="false">(C7-C8)/C8</f>
-        <v>0.0196834843010035</v>
+        <v>0.105385578555706</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B9" s="20" t="n">
-        <v>47318050</v>
+        <v>47400798</v>
       </c>
       <c r="C9" s="20" t="n">
-        <v>5241278</v>
+        <v>5402702</v>
       </c>
       <c r="D9" s="24" t="n">
         <f aca="false">(C9/B9)</f>
-        <v>0.110766990609292</v>
+        <v>0.11397913596307</v>
       </c>
       <c r="E9" s="23" t="n">
         <f aca="false">B8-B9</f>
-        <v>82748</v>
+        <v>85929</v>
       </c>
       <c r="F9" s="25" t="n">
         <f aca="false">(B8-B9)/B9</f>
-        <v>0.00174876183612807</v>
+        <v>0.00181281758167869</v>
       </c>
       <c r="G9" s="23" t="n">
         <f aca="false">C8-C9</f>
-        <v>161424</v>
+        <v>106344</v>
       </c>
       <c r="H9" s="25" t="n">
         <f aca="false">(C8-C9)/C9</f>
-        <v>0.0307985953044277</v>
+        <v>0.0196834843010035</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B10" s="20" t="n">
-        <v>46918951</v>
+        <v>47318050</v>
       </c>
       <c r="C10" s="20" t="n">
-        <v>4850762</v>
+        <v>5241278</v>
       </c>
       <c r="D10" s="24" t="n">
         <f aca="false">(C10/B10)</f>
-        <v>0.10338598576085</v>
+        <v>0.110766990609292</v>
       </c>
       <c r="E10" s="23" t="n">
         <f aca="false">B9-B10</f>
-        <v>399099</v>
+        <v>82748</v>
       </c>
       <c r="F10" s="25" t="n">
         <f aca="false">(B9-B10)/B10</f>
-        <v>0.00850613646498618</v>
+        <v>0.00174876183612807</v>
       </c>
       <c r="G10" s="23" t="n">
         <f aca="false">C9-C10</f>
-        <v>390516</v>
+        <v>161424</v>
       </c>
       <c r="H10" s="25" t="n">
         <f aca="false">(C9-C10)/C10</f>
-        <v>0.0805061142970939</v>
+        <v>0.0307985953044277</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B11" s="20" t="n">
-        <v>46645070</v>
+        <v>46918951</v>
       </c>
       <c r="C11" s="20" t="n">
-        <v>4577322</v>
+        <v>4850762</v>
       </c>
       <c r="D11" s="24" t="n">
         <f aca="false">(C11/B11)</f>
-        <v>0.0981308850002798</v>
+        <v>0.10338598576085</v>
       </c>
       <c r="E11" s="23" t="n">
         <f aca="false">B10-B11</f>
-        <v>273881</v>
+        <v>399099</v>
       </c>
       <c r="F11" s="25" t="n">
         <f aca="false">(B10-B11)/B11</f>
-        <v>0.00587159586211362</v>
+        <v>0.00850613646498618</v>
       </c>
       <c r="G11" s="23" t="n">
         <f aca="false">C10-C11</f>
-        <v>273440</v>
+        <v>390516</v>
       </c>
       <c r="H11" s="25" t="n">
         <f aca="false">(C10-C11)/C11</f>
-        <v>0.0597379865344846</v>
+        <v>0.0805061142970939</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B12" s="20" t="n">
-        <v>46497393</v>
+        <v>46645070</v>
       </c>
       <c r="C12" s="20" t="n">
-        <v>4417653</v>
+        <v>4577322</v>
       </c>
       <c r="D12" s="24" t="n">
         <f aca="false">(C12/B12)</f>
-        <v>0.0950086169347172</v>
+        <v>0.0981308850002798</v>
       </c>
       <c r="E12" s="23" t="n">
         <f aca="false">B11-B12</f>
-        <v>147677</v>
+        <v>273881</v>
       </c>
       <c r="F12" s="25" t="n">
         <f aca="false">(B11-B12)/B12</f>
-        <v>0.00317602752481198</v>
+        <v>0.00587159586211362</v>
       </c>
       <c r="G12" s="23" t="n">
         <f aca="false">C11-C12</f>
-        <v>159669</v>
+        <v>273440</v>
       </c>
       <c r="H12" s="25" t="n">
         <f aca="false">(C11-C12)/C12</f>
-        <v>0.0361434001267189</v>
+        <v>0.0597379865344846</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B13" s="20" t="n">
-        <v>46418884</v>
+        <v>46497393</v>
       </c>
       <c r="C13" s="20" t="n">
-        <v>4419334</v>
+        <v>4417653</v>
       </c>
       <c r="D13" s="24" t="n">
         <f aca="false">(C13/B13)</f>
-        <v>0.0952055202361177</v>
+        <v>0.0950086169347172</v>
       </c>
       <c r="E13" s="23" t="n">
         <f aca="false">B12-B13</f>
-        <v>78509</v>
+        <v>147677</v>
       </c>
       <c r="F13" s="25" t="n">
         <f aca="false">(B12-B13)/B13</f>
-        <v>0.00169131597390407</v>
+        <v>0.00317602752481198</v>
       </c>
       <c r="G13" s="23" t="n">
         <f aca="false">C12-C13</f>
-        <v>-1681</v>
+        <v>159669</v>
       </c>
       <c r="H13" s="25" t="n">
         <f aca="false">(C12-C13)/C13</f>
-        <v>-0.000380374056362339</v>
+        <v>0.0361434001267189</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B14" s="20" t="n">
-        <v>46425722</v>
+        <v>46418884</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>4453985</v>
+        <v>4419334</v>
       </c>
       <c r="D14" s="24" t="n">
         <f aca="false">(C14/B14)</f>
-        <v>0.0959378725440177</v>
+        <v>0.0952055202361177</v>
       </c>
       <c r="E14" s="23" t="n">
         <f aca="false">B13-B14</f>
-        <v>-6838</v>
+        <v>78509</v>
       </c>
       <c r="F14" s="25" t="n">
         <f aca="false">(B13-B14)/B14</f>
-        <v>-0.00014728903946825</v>
+        <v>0.00169131597390407</v>
       </c>
       <c r="G14" s="23" t="n">
         <f aca="false">C13-C14</f>
-        <v>-34651</v>
+        <v>-1681</v>
       </c>
       <c r="H14" s="25" t="n">
         <f aca="false">(C13-C14)/C14</f>
-        <v>-0.0077797747410465</v>
+        <v>-0.000380374056362339</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B15" s="20" t="n">
-        <v>46495744</v>
+        <v>46425722</v>
       </c>
       <c r="C15" s="20" t="n">
-        <v>4676352</v>
+        <v>4453985</v>
       </c>
       <c r="D15" s="24" t="n">
         <f aca="false">(C15/B15)</f>
-        <v>0.100575915077303</v>
+        <v>0.0959378725440177</v>
       </c>
       <c r="E15" s="23" t="n">
         <f aca="false">B14-B15</f>
-        <v>-70022</v>
+        <v>-6838</v>
       </c>
       <c r="F15" s="25" t="n">
         <f aca="false">(B14-B15)/B15</f>
-        <v>-0.00150598730068713</v>
+        <v>-0.00014728903946825</v>
       </c>
       <c r="G15" s="23" t="n">
         <f aca="false">C14-C15</f>
-        <v>-222367</v>
+        <v>-34651</v>
       </c>
       <c r="H15" s="25" t="n">
         <f aca="false">(C14-C15)/C15</f>
-        <v>-0.0475513819318991</v>
+        <v>-0.0077797747410465</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B16" s="20" t="n">
-        <v>46712650</v>
+        <v>46495744</v>
       </c>
       <c r="C16" s="20" t="n">
-        <v>5064584</v>
+        <v>4676352</v>
       </c>
       <c r="D16" s="24" t="n">
         <f aca="false">(C16/B16)</f>
-        <v>0.108419967610487</v>
+        <v>0.100575915077303</v>
       </c>
       <c r="E16" s="23" t="n">
         <f aca="false">B15-B16</f>
-        <v>-216906</v>
+        <v>-70022</v>
       </c>
       <c r="F16" s="25" t="n">
         <f aca="false">(B15-B16)/B16</f>
-        <v>-0.00464341029678256</v>
+        <v>-0.00150598730068713</v>
       </c>
       <c r="G16" s="23" t="n">
         <f aca="false">C15-C16</f>
-        <v>-388232</v>
+        <v>-222367</v>
       </c>
       <c r="H16" s="25" t="n">
         <f aca="false">(C15-C16)/C16</f>
-        <v>-0.0766562465939947</v>
+        <v>-0.0475513819318991</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B17" s="20" t="n">
-        <v>46818216</v>
+        <v>46712650</v>
       </c>
       <c r="C17" s="20" t="n">
-        <v>5236030</v>
+        <v>5064584</v>
       </c>
       <c r="D17" s="24" t="n">
         <f aca="false">(C17/B17)</f>
-        <v>0.111837452328384</v>
+        <v>0.108419967610487</v>
       </c>
       <c r="E17" s="23" t="n">
         <f aca="false">B16-B17</f>
-        <v>-105566</v>
+        <v>-216906</v>
       </c>
       <c r="F17" s="25" t="n">
         <f aca="false">(B16-B17)/B17</f>
-        <v>-0.00225480612076291</v>
+        <v>-0.00464341029678256</v>
       </c>
       <c r="G17" s="23" t="n">
         <f aca="false">C16-C17</f>
-        <v>-171446</v>
+        <v>-388232</v>
       </c>
       <c r="H17" s="25" t="n">
         <f aca="false">(C16-C17)/C17</f>
-        <v>-0.0327435098729381</v>
+        <v>-0.0766562465939947</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B18" s="20" t="n">
-        <v>46667175</v>
+        <v>46818216</v>
       </c>
       <c r="C18" s="20" t="n">
-        <v>5312440</v>
+        <v>5236030</v>
       </c>
       <c r="D18" s="24" t="n">
         <f aca="false">(C18/B18)</f>
-        <v>0.113836759992436</v>
+        <v>0.111837452328384</v>
       </c>
       <c r="E18" s="23" t="n">
         <f aca="false">B17-B18</f>
-        <v>151041</v>
+        <v>-105566</v>
       </c>
       <c r="F18" s="25" t="n">
         <f aca="false">(B17-B18)/B18</f>
-        <v>0.00323655760178327</v>
+        <v>-0.00225480612076291</v>
       </c>
       <c r="G18" s="23" t="n">
         <f aca="false">C17-C18</f>
-        <v>-76410</v>
+        <v>-171446</v>
       </c>
       <c r="H18" s="25" t="n">
         <f aca="false">(C17-C18)/C18</f>
-        <v>-0.0143832212693226</v>
+        <v>-0.0327435098729381</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B19" s="20" t="n">
-        <v>46486621</v>
+        <v>46667175</v>
       </c>
       <c r="C19" s="20" t="n">
-        <v>5402579</v>
+        <v>5312440</v>
       </c>
       <c r="D19" s="24" t="n">
         <f aca="false">(C19/B19)</f>
-        <v>0.116217932897295</v>
+        <v>0.113836759992436</v>
       </c>
       <c r="E19" s="23" t="n">
         <f aca="false">B18-B19</f>
-        <v>180554</v>
+        <v>151041</v>
       </c>
       <c r="F19" s="25" t="n">
         <f aca="false">(B18-B19)/B19</f>
-        <v>0.00388399922635805</v>
+        <v>0.00323655760178327</v>
       </c>
       <c r="G19" s="23" t="n">
         <f aca="false">C18-C19</f>
-        <v>-90139</v>
+        <v>-76410</v>
       </c>
       <c r="H19" s="25" t="n">
         <f aca="false">(C18-C19)/C19</f>
-        <v>-0.016684439042909</v>
+        <v>-0.0143832212693226</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B20" s="20" t="n">
-        <v>46239271</v>
+        <v>46486621</v>
       </c>
       <c r="C20" s="20" t="n">
-        <v>5386659</v>
+        <v>5402579</v>
       </c>
       <c r="D20" s="24" t="n">
         <f aca="false">(C20/B20)</f>
-        <v>0.116495327099772</v>
+        <v>0.116217932897295</v>
       </c>
       <c r="E20" s="23" t="n">
         <f aca="false">B19-B20</f>
-        <v>247350</v>
+        <v>180554</v>
       </c>
       <c r="F20" s="25" t="n">
         <f aca="false">(B19-B20)/B20</f>
-        <v>0.00534934904142412</v>
+        <v>0.00388399922635805</v>
       </c>
       <c r="G20" s="23" t="n">
         <f aca="false">C19-C20</f>
-        <v>15920</v>
+        <v>-90139</v>
       </c>
       <c r="H20" s="25" t="n">
         <f aca="false">(C19-C20)/C20</f>
-        <v>0.00295544975094952</v>
+        <v>-0.016684439042909</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B21" s="20" t="n">
-        <v>45668938</v>
+        <v>46239271</v>
       </c>
       <c r="C21" s="20" t="n">
-        <v>5086295</v>
+        <v>5386659</v>
       </c>
       <c r="D21" s="24" t="n">
         <f aca="false">(C21/B21)</f>
-        <v>0.111373183234521</v>
+        <v>0.116495327099772</v>
       </c>
       <c r="E21" s="23" t="n">
         <f aca="false">B20-B21</f>
-        <v>570333</v>
+        <v>247350</v>
       </c>
       <c r="F21" s="25" t="n">
         <f aca="false">(B20-B21)/B21</f>
-        <v>0.0124884226561169</v>
+        <v>0.00534934904142412</v>
       </c>
       <c r="G21" s="23" t="n">
         <f aca="false">C20-C21</f>
-        <v>300364</v>
+        <v>15920</v>
       </c>
       <c r="H21" s="25" t="n">
         <f aca="false">(C20-C21)/C21</f>
-        <v>0.0590535940207951</v>
+        <v>0.00295544975094952</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B22" s="20" t="n">
-        <v>44784659</v>
+        <v>45668938</v>
       </c>
       <c r="C22" s="20" t="n">
-        <v>4449434</v>
+        <v>5086295</v>
       </c>
       <c r="D22" s="24" t="n">
         <f aca="false">(C22/B22)</f>
-        <v>0.0993517445337699</v>
+        <v>0.111373183234521</v>
       </c>
       <c r="E22" s="23" t="n">
         <f aca="false">B21-B22</f>
-        <v>884279</v>
+        <v>570333</v>
       </c>
       <c r="F22" s="25" t="n">
         <f aca="false">(B21-B22)/B22</f>
-        <v>0.0197451319211786</v>
+        <v>0.0124884226561169</v>
       </c>
       <c r="G22" s="23" t="n">
         <f aca="false">C21-C22</f>
-        <v>636861</v>
+        <v>300364</v>
       </c>
       <c r="H22" s="25" t="n">
         <f aca="false">(C21-C22)/C22</f>
-        <v>0.143133036696353</v>
+        <v>0.0590535940207951</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B23" s="20" t="n">
-        <v>44009969</v>
+        <v>44784659</v>
       </c>
       <c r="C23" s="20" t="n">
-        <v>3930916</v>
+        <v>4449434</v>
       </c>
       <c r="D23" s="24" t="n">
         <f aca="false">(C23/B23)</f>
-        <v>0.0893187632102172</v>
+        <v>0.0993517445337699</v>
       </c>
       <c r="E23" s="23" t="n">
         <f aca="false">B22-B23</f>
-        <v>774690</v>
+        <v>884279</v>
       </c>
       <c r="F23" s="25" t="n">
         <f aca="false">(B22-B23)/B23</f>
-        <v>0.0176026027193975</v>
+        <v>0.0197451319211786</v>
       </c>
       <c r="G23" s="23" t="n">
         <f aca="false">C22-C23</f>
-        <v>518518</v>
+        <v>636861</v>
       </c>
       <c r="H23" s="25" t="n">
         <f aca="false">(C22-C23)/C23</f>
-        <v>0.131907677498069</v>
+        <v>0.143133036696353</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B24" s="20" t="n">
-        <v>43296335</v>
+        <v>44009969</v>
       </c>
       <c r="C24" s="20" t="n">
-        <v>3430204</v>
+        <v>3930916</v>
       </c>
       <c r="D24" s="24" t="n">
         <f aca="false">(C24/B24)</f>
-        <v>0.0792261977832535</v>
+        <v>0.0893187632102172</v>
       </c>
       <c r="E24" s="23" t="n">
         <f aca="false">B23-B24</f>
-        <v>713634</v>
+        <v>774690</v>
       </c>
       <c r="F24" s="25" t="n">
         <f aca="false">(B23-B24)/B24</f>
-        <v>0.0164825498509285</v>
+        <v>0.0176026027193975</v>
       </c>
       <c r="G24" s="23" t="n">
         <f aca="false">C23-C24</f>
-        <v>500712</v>
+        <v>518518</v>
       </c>
       <c r="H24" s="25" t="n">
         <f aca="false">(C23-C24)/C24</f>
-        <v>0.145971493240635</v>
+        <v>0.131907677498069</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>43296335</v>
+      </c>
+      <c r="C25" s="20" t="n">
+        <v>3430204</v>
+      </c>
+      <c r="D25" s="24" t="n">
+        <f aca="false">(C25/B25)</f>
+        <v>0.0792261977832535</v>
+      </c>
+      <c r="E25" s="23" t="n">
+        <f aca="false">B24-B25</f>
+        <v>713634</v>
+      </c>
+      <c r="F25" s="25" t="n">
+        <f aca="false">(B24-B25)/B25</f>
+        <v>0.0164825498509285</v>
+      </c>
+      <c r="G25" s="23" t="n">
+        <f aca="false">C24-C25</f>
+        <v>500712</v>
+      </c>
+      <c r="H25" s="25" t="n">
+        <f aca="false">(C24-C25)/C25</f>
+        <v>0.145971493240635</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="20" t="n">
+      <c r="B26" s="20" t="n">
         <v>42547454</v>
       </c>
-      <c r="C25" s="20"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="23"/>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="23"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
+      <c r="C26" s="20"/>
       <c r="D26" s="23"/>
       <c r="E26" s="23"/>
       <c r="F26" s="23"/>
       <c r="G26" s="23"/>
       <c r="H26" s="23"/>
     </row>
-    <row r="28" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8"/>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>14</v>
-      </c>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="23"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>250</v>
+        <v>13</v>
       </c>
       <c r="B31" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="s">
+      <c r="B32" s="1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B34" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="1" t="s">
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="1" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:E34"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Página &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>